<commit_message>
Clear incorrect profile URLs from company account rows
The scraper wasn't built to handle company account posts — it grabbed
random profiles (commenters, suggestions) instead of recognizing the
post was from a company page. Cleared 12 wrong mappings.

https://claude.ai/code/session_01TxBD8Aq88yMmNXwZYTVy7v
</commit_message>
<xml_diff>
--- a/New - Customer influencer reachouts.xlsx
+++ b/New - Customer influencer reachouts.xlsx
@@ -453,7 +453,7 @@
           <t>Sent</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/bettina-i-berntsen</t>
         </is>
@@ -475,7 +475,7 @@
           <t>Sent</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/pontus-lindgren-aa7538141</t>
         </is>
@@ -497,7 +497,7 @@
           <t>connected</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/jos-van-der-kooij</t>
         </is>
@@ -519,7 +519,7 @@
           <t>sent</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/andrewjohnwalls</t>
         </is>
@@ -541,7 +541,7 @@
           <t>Sent</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/keeswolters</t>
         </is>
@@ -563,7 +563,7 @@
           <t>Sent</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -585,7 +585,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -607,7 +607,7 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -629,7 +629,7 @@
           <t>connected</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/shawn-gordon-37b9916</t>
         </is>
@@ -651,7 +651,7 @@
           <t>sent</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/aira-mongush</t>
         </is>
@@ -673,7 +673,7 @@
           <t>skip</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/rewillis</t>
         </is>
@@ -695,7 +695,7 @@
           <t>sent</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/inkenthomas</t>
         </is>
@@ -717,7 +717,7 @@
           <t>sent</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/vickranth-muthulingaperumal-352664224</t>
         </is>
@@ -739,7 +739,7 @@
           <t>skip</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/brintha-kumaresan</t>
         </is>
@@ -761,7 +761,7 @@
           <t>sent</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/colin-a-campbell</t>
         </is>
@@ -783,7 +783,7 @@
           <t>sent</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/peterschouba</t>
         </is>
@@ -805,7 +805,7 @@
           <t>skip</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/mefuller</t>
         </is>
@@ -827,7 +827,7 @@
           <t>sent</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/raghunathv</t>
         </is>
@@ -849,9 +849,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/nalinpradeep</t>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
           <t>sent</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/peterpcooper</t>
         </is>
@@ -893,9 +893,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/lindseyamcdonald29</t>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -915,9 +915,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/kevin-healey-0a815112</t>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
           <t>skip</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/kev-wheatley</t>
         </is>
@@ -959,9 +959,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/iallen1</t>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -981,9 +981,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/teodorum</t>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -1003,9 +1003,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/nagarjun-reddy</t>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -1047,7 +1047,7 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -1069,9 +1069,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/usman-shahid-0985ab262</t>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -1113,9 +1113,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/abiodun-adeyanju-5488a821b</t>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -1157,7 +1157,7 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -1179,9 +1179,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/arthur-castillo</t>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -1201,9 +1201,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/chris-koehnecke-3619333</t>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -1223,9 +1223,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/alysilver</t>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>(no profile found)</t>
         </is>
@@ -1267,9 +1267,9 @@
           <t>company ac</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/anirudh-w</t>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>(company account)</t>
         </is>
       </c>
     </row>

</xml_diff>